<commit_message>
feat: update bookshelf visuals and align docs
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/src/data/dishes.xlsx
+++ b/src/data/dishes.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="21600" windowHeight="10455"/>
+    <workbookView windowWidth="11130" windowHeight="10455"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -2094,7 +2094,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:H1 A2:B27 D2:D27 G2:G25 A28:H28" numberStoredAsText="1"/>
+    <ignoredError sqref="A28:H28 G2:G25 D6 D8:D10 D12 D15 D18:D22 D26:D27 A2:B22 B23 A24:B26 B27 A1:H1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat: refine map panel data and tooling
Made-with: Cursor
</commit_message>
<xml_diff>
--- a/src/data/dishes.xlsx
+++ b/src/data/dishes.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
   <bookViews>
-    <workbookView windowWidth="11130" windowHeight="10455"/>
+    <workbookView windowWidth="21600" windowHeight="10455"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -27,30 +27,36 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="179" uniqueCount="62">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="207" uniqueCount="64">
   <si>
     <t>store_name_zh</t>
   </si>
   <si>
+    <t>store_name_en</t>
+  </si>
+  <si>
     <t>store_name_local</t>
   </si>
   <si>
     <t>city_en</t>
   </si>
   <si>
-    <t>name_zh</t>
-  </si>
-  <si>
-    <t>name_en</t>
-  </si>
-  <si>
-    <t>name_local</t>
+    <t>dish_name_zh</t>
+  </si>
+  <si>
+    <t>dish_name_en</t>
+  </si>
+  <si>
+    <t>dish_name_local</t>
   </si>
   <si>
     <t>price</t>
   </si>
   <si>
     <t>taste</t>
+  </si>
+  <si>
+    <t>note</t>
   </si>
   <si>
     <t>仙生生寿司专门店(中山店)</t>
@@ -1372,20 +1378,21 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:etc="http://www.wps.cn/officeDocument/2017/etCustomData">
   <sheetPr/>
-  <dimension ref="A1:H28"/>
-  <sheetFormatPr defaultColWidth="9.02654867256637" defaultRowHeight="13.5" outlineLevelCol="7"/>
+  <dimension ref="A1:J28"/>
+  <sheetFormatPr defaultColWidth="9.02654867256637" defaultRowHeight="13.5"/>
   <cols>
     <col min="1" max="1" width="41.5752212389381" customWidth="1"/>
-    <col min="2" max="2" width="18.3893805309735" customWidth="1"/>
-    <col min="3" max="3" width="8.53097345132743" customWidth="1"/>
-    <col min="4" max="4" width="22.0796460176991" customWidth="1"/>
-    <col min="5" max="5" width="8.53097345132743" customWidth="1"/>
-    <col min="6" max="6" width="11.7256637168142" customWidth="1"/>
-    <col min="7" max="7" width="6.53097345132743" style="1" customWidth="1"/>
-    <col min="8" max="8" width="9.30088495575221" customWidth="1"/>
+    <col min="2" max="2" width="15.0619469026549" customWidth="1"/>
+    <col min="3" max="3" width="18.3893805309735" customWidth="1"/>
+    <col min="4" max="4" width="8.53097345132743" customWidth="1"/>
+    <col min="5" max="5" width="22.0796460176991" customWidth="1"/>
+    <col min="6" max="6" width="13.929203539823" customWidth="1"/>
+    <col min="7" max="7" width="17.3274336283186" customWidth="1"/>
+    <col min="8" max="8" width="6.53097345132743" style="1" customWidth="1"/>
+    <col min="9" max="9" width="9.30088495575221" style="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8">
+    <row r="1" spans="1:10">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
@@ -1404,697 +1411,781 @@
       <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="2" spans="1:8">
+      <c r="I1" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="J1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10">
       <c r="A2" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B2" t="s">
+        <v>11</v>
+      </c>
+      <c r="C2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E2" t="s">
+        <v>13</v>
+      </c>
+      <c r="F2" t="s">
+        <v>11</v>
+      </c>
+      <c r="G2" t="s">
+        <v>11</v>
+      </c>
+      <c r="H2" s="1" t="s">
+        <v>14</v>
+      </c>
+      <c r="I2" s="1">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10">
+      <c r="A3" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>11</v>
+      </c>
+      <c r="C3" t="s">
+        <v>11</v>
+      </c>
+      <c r="D3" t="s">
+        <v>12</v>
+      </c>
+      <c r="E3" t="s">
+        <v>15</v>
+      </c>
+      <c r="F3" t="s">
+        <v>11</v>
+      </c>
+      <c r="G3" t="s">
+        <v>11</v>
+      </c>
+      <c r="H3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="I3" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10">
+      <c r="A4" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>11</v>
+      </c>
+      <c r="C4" t="s">
+        <v>11</v>
+      </c>
+      <c r="D4" t="s">
+        <v>12</v>
+      </c>
+      <c r="E4" t="s">
+        <v>17</v>
+      </c>
+      <c r="F4" t="s">
+        <v>11</v>
+      </c>
+      <c r="G4" t="s">
+        <v>11</v>
+      </c>
+      <c r="H4" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="I4" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="5" spans="1:10">
+      <c r="A5" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5" t="s">
+        <v>11</v>
+      </c>
+      <c r="D5" t="s">
+        <v>12</v>
+      </c>
+      <c r="E5" t="s">
+        <v>19</v>
+      </c>
+      <c r="F5" t="s">
+        <v>11</v>
+      </c>
+      <c r="G5" t="s">
+        <v>11</v>
+      </c>
+      <c r="H5" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="I5" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" spans="1:10">
+      <c r="A6" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B6" t="s">
+        <v>11</v>
+      </c>
+      <c r="C6" t="s">
+        <v>11</v>
+      </c>
+      <c r="D6" t="s">
+        <v>12</v>
+      </c>
+      <c r="E6" t="s">
+        <v>21</v>
+      </c>
+      <c r="F6" t="s">
+        <v>11</v>
+      </c>
+      <c r="G6" t="s">
+        <v>11</v>
+      </c>
+      <c r="H6" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="I6" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10">
+      <c r="A7" s="3" t="s">
+        <v>10</v>
+      </c>
+      <c r="B7" t="s">
+        <v>11</v>
+      </c>
+      <c r="C7" t="s">
+        <v>11</v>
+      </c>
+      <c r="D7" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" t="s">
+        <v>23</v>
+      </c>
+      <c r="F7" t="s">
+        <v>11</v>
+      </c>
+      <c r="G7" t="s">
+        <v>11</v>
+      </c>
+      <c r="H7" s="1" t="s">
+        <v>24</v>
+      </c>
+      <c r="I7" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10">
+      <c r="A8" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B8" t="s">
+        <v>11</v>
+      </c>
+      <c r="C8" t="s">
+        <v>11</v>
+      </c>
+      <c r="D8" t="s">
+        <v>12</v>
+      </c>
+      <c r="E8" t="s">
+        <v>26</v>
+      </c>
+      <c r="F8" t="s">
+        <v>11</v>
+      </c>
+      <c r="G8" t="s">
+        <v>11</v>
+      </c>
+      <c r="H8" s="1" t="s">
+        <v>27</v>
+      </c>
+      <c r="I8" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10">
+      <c r="A9" s="3" t="s">
+        <v>25</v>
+      </c>
+      <c r="B9" t="s">
+        <v>11</v>
+      </c>
+      <c r="C9" t="s">
+        <v>11</v>
+      </c>
+      <c r="D9" t="s">
+        <v>12</v>
+      </c>
+      <c r="E9" t="s">
+        <v>28</v>
+      </c>
+      <c r="F9" t="s">
+        <v>11</v>
+      </c>
+      <c r="G9" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="I9" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10">
+      <c r="A10" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10" t="s">
+        <v>11</v>
+      </c>
+      <c r="D10" t="s">
+        <v>12</v>
+      </c>
+      <c r="E10" t="s">
+        <v>31</v>
+      </c>
+      <c r="F10" t="s">
+        <v>11</v>
+      </c>
+      <c r="G10" t="s">
+        <v>11</v>
+      </c>
+      <c r="H10" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="I10" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10">
+      <c r="A11" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B11" t="s">
+        <v>11</v>
+      </c>
+      <c r="C11" t="s">
+        <v>11</v>
+      </c>
+      <c r="D11" t="s">
+        <v>12</v>
+      </c>
+      <c r="E11" t="s">
+        <v>33</v>
+      </c>
+      <c r="F11" t="s">
+        <v>11</v>
+      </c>
+      <c r="G11" t="s">
+        <v>11</v>
+      </c>
+      <c r="H11" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="I11" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="12" spans="1:10">
+      <c r="A12" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B12" t="s">
+        <v>11</v>
+      </c>
+      <c r="C12" t="s">
+        <v>11</v>
+      </c>
+      <c r="D12" t="s">
+        <v>12</v>
+      </c>
+      <c r="E12" t="s">
+        <v>35</v>
+      </c>
+      <c r="F12" t="s">
+        <v>11</v>
+      </c>
+      <c r="G12" t="s">
+        <v>11</v>
+      </c>
+      <c r="H12" s="1" t="s">
+        <v>36</v>
+      </c>
+      <c r="I12" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="13" customFormat="1" spans="1:10">
+      <c r="A13" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13" t="s">
+        <v>11</v>
+      </c>
+      <c r="D13" t="s">
+        <v>12</v>
+      </c>
+      <c r="E13" t="s">
+        <v>37</v>
+      </c>
+      <c r="F13" t="s">
+        <v>11</v>
+      </c>
+      <c r="G13" t="s">
+        <v>11</v>
+      </c>
+      <c r="H13" s="1" t="s">
+        <v>38</v>
+      </c>
+      <c r="I13" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="14" spans="1:10">
+      <c r="A14" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B14" t="s">
+        <v>11</v>
+      </c>
+      <c r="C14" t="s">
+        <v>11</v>
+      </c>
+      <c r="D14" t="s">
+        <v>12</v>
+      </c>
+      <c r="E14" t="s">
+        <v>39</v>
+      </c>
+      <c r="F14" t="s">
+        <v>11</v>
+      </c>
+      <c r="G14" t="s">
+        <v>11</v>
+      </c>
+      <c r="H14" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="I14" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" spans="1:10">
+      <c r="A15" s="3" t="s">
+        <v>30</v>
+      </c>
+      <c r="B15" t="s">
+        <v>11</v>
+      </c>
+      <c r="C15" t="s">
+        <v>11</v>
+      </c>
+      <c r="D15" t="s">
+        <v>12</v>
+      </c>
+      <c r="E15" t="s">
+        <v>41</v>
+      </c>
+      <c r="F15" t="s">
+        <v>11</v>
+      </c>
+      <c r="G15" t="s">
+        <v>11</v>
+      </c>
+      <c r="H15" s="1">
         <v>8</v>
       </c>
-      <c r="B2" t="s">
-        <v>9</v>
-      </c>
-      <c r="C2" t="s">
-        <v>10</v>
-      </c>
-      <c r="D2" t="s">
-        <v>11</v>
-      </c>
-      <c r="E2" t="s">
-        <v>9</v>
-      </c>
-      <c r="F2" t="s">
-        <v>9</v>
-      </c>
-      <c r="G2" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="H2">
+      <c r="I15" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="16" spans="1:10">
+      <c r="A16" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16" t="s">
+        <v>11</v>
+      </c>
+      <c r="D16" t="s">
+        <v>12</v>
+      </c>
+      <c r="E16" t="s">
+        <v>43</v>
+      </c>
+      <c r="F16" t="s">
+        <v>11</v>
+      </c>
+      <c r="G16" t="s">
+        <v>11</v>
+      </c>
+      <c r="H16" s="1">
+        <v>17.8</v>
+      </c>
+      <c r="I16" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="B17" t="s">
+        <v>11</v>
+      </c>
+      <c r="C17" t="s">
+        <v>11</v>
+      </c>
+      <c r="D17" t="s">
+        <v>12</v>
+      </c>
+      <c r="E17" t="s">
+        <v>44</v>
+      </c>
+      <c r="F17" t="s">
+        <v>11</v>
+      </c>
+      <c r="G17" t="s">
+        <v>11</v>
+      </c>
+      <c r="H17" s="1">
+        <v>14.8</v>
+      </c>
+      <c r="I17" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B18" t="s">
+        <v>11</v>
+      </c>
+      <c r="C18" t="s">
+        <v>11</v>
+      </c>
+      <c r="D18" t="s">
+        <v>12</v>
+      </c>
+      <c r="E18" t="s">
+        <v>46</v>
+      </c>
+      <c r="F18" t="s">
+        <v>11</v>
+      </c>
+      <c r="G18" t="s">
+        <v>11</v>
+      </c>
+      <c r="H18" s="1">
+        <v>49</v>
+      </c>
+      <c r="I18" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="3" t="s">
+        <v>45</v>
+      </c>
+      <c r="B19" t="s">
+        <v>11</v>
+      </c>
+      <c r="C19" t="s">
+        <v>11</v>
+      </c>
+      <c r="D19" t="s">
+        <v>12</v>
+      </c>
+      <c r="E19" t="s">
+        <v>47</v>
+      </c>
+      <c r="F19" t="s">
+        <v>11</v>
+      </c>
+      <c r="G19" t="s">
+        <v>11</v>
+      </c>
+      <c r="H19" s="1">
+        <v>12</v>
+      </c>
+      <c r="I19" s="1">
+        <v>1</v>
+      </c>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="3" t="s">
+        <v>48</v>
+      </c>
+      <c r="B20" t="s">
+        <v>11</v>
+      </c>
+      <c r="C20" t="s">
+        <v>11</v>
+      </c>
+      <c r="D20" t="s">
+        <v>12</v>
+      </c>
+      <c r="E20" t="s">
+        <v>49</v>
+      </c>
+      <c r="F20" t="s">
+        <v>11</v>
+      </c>
+      <c r="G20" t="s">
+        <v>11</v>
+      </c>
+      <c r="H20" s="1">
+        <v>15</v>
+      </c>
+      <c r="I20" s="1">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" t="s">
+        <v>50</v>
+      </c>
+      <c r="B21" t="s">
+        <v>11</v>
+      </c>
+      <c r="C21" t="s">
+        <v>11</v>
+      </c>
+      <c r="D21" t="s">
+        <v>12</v>
+      </c>
+      <c r="E21" t="s">
+        <v>51</v>
+      </c>
+      <c r="F21" t="s">
+        <v>11</v>
+      </c>
+      <c r="G21" t="s">
+        <v>11</v>
+      </c>
+      <c r="H21" s="1">
+        <v>17.2</v>
+      </c>
+      <c r="I21" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" t="s">
+        <v>50</v>
+      </c>
+      <c r="B22" t="s">
+        <v>11</v>
+      </c>
+      <c r="C22" t="s">
+        <v>11</v>
+      </c>
+      <c r="D22" t="s">
+        <v>12</v>
+      </c>
+      <c r="E22" t="s">
+        <v>52</v>
+      </c>
+      <c r="F22" t="s">
+        <v>11</v>
+      </c>
+      <c r="G22" t="s">
+        <v>11</v>
+      </c>
+      <c r="H22" s="1">
+        <v>21.3</v>
+      </c>
+      <c r="I22" s="1">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" t="s">
+        <v>53</v>
+      </c>
+      <c r="B23" t="s">
+        <v>11</v>
+      </c>
+      <c r="C23" t="s">
+        <v>11</v>
+      </c>
+      <c r="D23" t="s">
+        <v>12</v>
+      </c>
+      <c r="E23" t="s">
+        <v>54</v>
+      </c>
+      <c r="F23" t="s">
+        <v>11</v>
+      </c>
+      <c r="G23" t="s">
+        <v>11</v>
+      </c>
+      <c r="H23" s="1">
+        <v>42</v>
+      </c>
+      <c r="I23" s="1">
         <v>5</v>
       </c>
     </row>
-    <row r="3" spans="1:8">
-      <c r="A3" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B3" t="s">
-        <v>9</v>
-      </c>
-      <c r="C3" t="s">
-        <v>10</v>
-      </c>
-      <c r="D3" t="s">
-        <v>13</v>
-      </c>
-      <c r="E3" t="s">
-        <v>9</v>
-      </c>
-      <c r="F3" t="s">
-        <v>9</v>
-      </c>
-      <c r="G3" s="1" t="s">
-        <v>14</v>
-      </c>
-      <c r="H3">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="4" spans="1:8">
-      <c r="A4" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B4" t="s">
-        <v>9</v>
-      </c>
-      <c r="C4" t="s">
-        <v>10</v>
-      </c>
-      <c r="D4" t="s">
-        <v>15</v>
-      </c>
-      <c r="E4" t="s">
-        <v>9</v>
-      </c>
-      <c r="F4" t="s">
-        <v>9</v>
-      </c>
-      <c r="G4" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="H4">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="5" spans="1:8">
-      <c r="A5" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B5" t="s">
-        <v>9</v>
-      </c>
-      <c r="C5" t="s">
-        <v>10</v>
-      </c>
-      <c r="D5" t="s">
-        <v>17</v>
-      </c>
-      <c r="E5" t="s">
-        <v>9</v>
-      </c>
-      <c r="F5" t="s">
-        <v>9</v>
-      </c>
-      <c r="G5" s="1" t="s">
-        <v>18</v>
-      </c>
-      <c r="H5">
+    <row r="24" spans="1:9">
+      <c r="A24" t="s">
+        <v>55</v>
+      </c>
+      <c r="B24" t="s">
+        <v>11</v>
+      </c>
+      <c r="C24" t="s">
+        <v>11</v>
+      </c>
+      <c r="D24" t="s">
+        <v>12</v>
+      </c>
+      <c r="E24" t="s">
+        <v>56</v>
+      </c>
+      <c r="F24" t="s">
+        <v>11</v>
+      </c>
+      <c r="G24" t="s">
+        <v>11</v>
+      </c>
+      <c r="H24" s="1">
+        <v>66</v>
+      </c>
+      <c r="I24" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="6" spans="1:8">
-      <c r="A6" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B6" t="s">
-        <v>9</v>
-      </c>
-      <c r="C6" t="s">
-        <v>10</v>
-      </c>
-      <c r="D6" t="s">
-        <v>19</v>
-      </c>
-      <c r="E6" t="s">
-        <v>9</v>
-      </c>
-      <c r="F6" t="s">
-        <v>9</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>20</v>
-      </c>
-      <c r="H6">
+    <row r="25" spans="1:9">
+      <c r="A25" t="s">
+        <v>57</v>
+      </c>
+      <c r="B25" t="s">
+        <v>11</v>
+      </c>
+      <c r="C25" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" t="s">
+        <v>58</v>
+      </c>
+      <c r="F25" t="s">
+        <v>11</v>
+      </c>
+      <c r="G25" t="s">
+        <v>11</v>
+      </c>
+      <c r="H25" s="1">
+        <v>35</v>
+      </c>
+      <c r="I25" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="7" spans="1:8">
-      <c r="A7" s="3" t="s">
-        <v>8</v>
-      </c>
-      <c r="B7" t="s">
-        <v>9</v>
-      </c>
-      <c r="C7" t="s">
-        <v>10</v>
-      </c>
-      <c r="D7" t="s">
-        <v>21</v>
-      </c>
-      <c r="E7" t="s">
-        <v>9</v>
-      </c>
-      <c r="F7" t="s">
-        <v>9</v>
-      </c>
-      <c r="G7" s="1" t="s">
-        <v>22</v>
-      </c>
-      <c r="H7">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="8" spans="1:8">
-      <c r="A8" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B8" t="s">
-        <v>9</v>
-      </c>
-      <c r="C8" t="s">
-        <v>10</v>
-      </c>
-      <c r="D8" t="s">
-        <v>24</v>
-      </c>
-      <c r="E8" t="s">
-        <v>9</v>
-      </c>
-      <c r="F8" t="s">
-        <v>9</v>
-      </c>
-      <c r="G8" s="1" t="s">
-        <v>25</v>
-      </c>
-      <c r="H8">
+    <row r="26" spans="1:9">
+      <c r="A26" t="s">
+        <v>59</v>
+      </c>
+      <c r="B26" t="s">
+        <v>11</v>
+      </c>
+      <c r="C26" t="s">
+        <v>11</v>
+      </c>
+      <c r="D26" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" t="s">
+        <v>60</v>
+      </c>
+      <c r="F26" t="s">
+        <v>11</v>
+      </c>
+      <c r="G26" t="s">
+        <v>11</v>
+      </c>
+      <c r="H26" s="1" t="s">
+        <v>61</v>
+      </c>
+      <c r="I26" s="1">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" t="s">
+        <v>59</v>
+      </c>
+      <c r="B27" t="s">
+        <v>11</v>
+      </c>
+      <c r="C27" t="s">
+        <v>11</v>
+      </c>
+      <c r="D27" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" t="s">
+        <v>62</v>
+      </c>
+      <c r="F27" t="s">
+        <v>11</v>
+      </c>
+      <c r="G27" t="s">
+        <v>11</v>
+      </c>
+      <c r="H27" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="I27" s="1">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="1:8">
-      <c r="A9" s="3" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" t="s">
-        <v>9</v>
-      </c>
-      <c r="C9" t="s">
-        <v>10</v>
-      </c>
-      <c r="D9" t="s">
-        <v>26</v>
-      </c>
-      <c r="E9" t="s">
-        <v>9</v>
-      </c>
-      <c r="F9" t="s">
-        <v>9</v>
-      </c>
-      <c r="G9" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="H9">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="10" spans="1:8">
-      <c r="A10" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B10" t="s">
-        <v>9</v>
-      </c>
-      <c r="C10" t="s">
-        <v>10</v>
-      </c>
-      <c r="D10" t="s">
-        <v>29</v>
-      </c>
-      <c r="E10" t="s">
-        <v>9</v>
-      </c>
-      <c r="F10" t="s">
-        <v>9</v>
-      </c>
-      <c r="G10" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="H10">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="11" spans="1:8">
-      <c r="A11" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B11" t="s">
-        <v>9</v>
-      </c>
-      <c r="C11" t="s">
-        <v>10</v>
-      </c>
-      <c r="D11" t="s">
-        <v>31</v>
-      </c>
-      <c r="E11" t="s">
-        <v>9</v>
-      </c>
-      <c r="F11" t="s">
-        <v>9</v>
-      </c>
-      <c r="G11" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="H11">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="12" spans="1:8">
-      <c r="A12" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B12" t="s">
-        <v>9</v>
-      </c>
-      <c r="C12" t="s">
-        <v>10</v>
-      </c>
-      <c r="D12" t="s">
-        <v>33</v>
-      </c>
-      <c r="E12" t="s">
-        <v>9</v>
-      </c>
-      <c r="F12" t="s">
-        <v>9</v>
-      </c>
-      <c r="G12" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="H12">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="13" customFormat="1" spans="1:8">
-      <c r="A13" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B13" t="s">
-        <v>9</v>
-      </c>
-      <c r="C13" t="s">
-        <v>10</v>
-      </c>
-      <c r="D13" t="s">
-        <v>35</v>
-      </c>
-      <c r="E13" t="s">
-        <v>9</v>
-      </c>
-      <c r="F13" t="s">
-        <v>9</v>
-      </c>
-      <c r="G13" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="H13">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="14" spans="1:8">
-      <c r="A14" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B14" t="s">
-        <v>9</v>
-      </c>
-      <c r="C14" t="s">
-        <v>10</v>
-      </c>
-      <c r="D14" t="s">
-        <v>37</v>
-      </c>
-      <c r="E14" t="s">
-        <v>9</v>
-      </c>
-      <c r="F14" t="s">
-        <v>9</v>
-      </c>
-      <c r="G14" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="H14">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="15" spans="1:8">
-      <c r="A15" s="3" t="s">
-        <v>28</v>
-      </c>
-      <c r="B15" t="s">
-        <v>9</v>
-      </c>
-      <c r="C15" t="s">
-        <v>10</v>
-      </c>
-      <c r="D15" t="s">
-        <v>39</v>
-      </c>
-      <c r="E15" t="s">
-        <v>9</v>
-      </c>
-      <c r="F15" t="s">
-        <v>9</v>
-      </c>
-      <c r="G15" s="1">
-        <v>8</v>
-      </c>
-      <c r="H15">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="16" spans="1:8">
-      <c r="A16" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B16" t="s">
-        <v>9</v>
-      </c>
-      <c r="C16" t="s">
-        <v>10</v>
-      </c>
-      <c r="D16" t="s">
-        <v>41</v>
-      </c>
-      <c r="E16" t="s">
-        <v>9</v>
-      </c>
-      <c r="F16" t="s">
-        <v>9</v>
-      </c>
-      <c r="G16" s="1">
-        <v>17.8</v>
-      </c>
-      <c r="H16">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="17" spans="1:8">
-      <c r="A17" s="3" t="s">
-        <v>40</v>
-      </c>
-      <c r="B17" t="s">
-        <v>9</v>
-      </c>
-      <c r="C17" t="s">
-        <v>10</v>
-      </c>
-      <c r="D17" t="s">
-        <v>42</v>
-      </c>
-      <c r="E17" t="s">
-        <v>9</v>
-      </c>
-      <c r="F17" t="s">
-        <v>9</v>
-      </c>
-      <c r="G17" s="1">
-        <v>14.8</v>
-      </c>
-      <c r="H17">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="18" spans="1:8">
-      <c r="A18" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B18" t="s">
-        <v>9</v>
-      </c>
-      <c r="C18" t="s">
-        <v>10</v>
-      </c>
-      <c r="D18" t="s">
-        <v>44</v>
-      </c>
-      <c r="E18" t="s">
-        <v>9</v>
-      </c>
-      <c r="F18" t="s">
-        <v>9</v>
-      </c>
-      <c r="G18" s="1">
-        <v>49</v>
-      </c>
-      <c r="H18">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="19" spans="1:8">
-      <c r="A19" s="3" t="s">
-        <v>43</v>
-      </c>
-      <c r="B19" t="s">
-        <v>9</v>
-      </c>
-      <c r="C19" t="s">
-        <v>10</v>
-      </c>
-      <c r="D19" t="s">
-        <v>45</v>
-      </c>
-      <c r="E19" t="s">
-        <v>9</v>
-      </c>
-      <c r="F19" t="s">
-        <v>9</v>
-      </c>
-      <c r="G19" s="1">
-        <v>12</v>
-      </c>
-      <c r="H19">
-        <v>1</v>
-      </c>
-    </row>
-    <row r="20" spans="1:8">
-      <c r="A20" s="3" t="s">
-        <v>46</v>
-      </c>
-      <c r="B20" t="s">
-        <v>9</v>
-      </c>
-      <c r="C20" t="s">
-        <v>10</v>
-      </c>
-      <c r="D20" t="s">
-        <v>47</v>
-      </c>
-      <c r="E20" t="s">
-        <v>9</v>
-      </c>
-      <c r="F20" t="s">
-        <v>9</v>
-      </c>
-      <c r="G20" s="1">
-        <v>15</v>
-      </c>
-      <c r="H20">
-        <v>4</v>
-      </c>
-    </row>
-    <row r="21" spans="1:8">
-      <c r="A21" t="s">
-        <v>48</v>
-      </c>
-      <c r="B21" t="s">
-        <v>9</v>
-      </c>
-      <c r="C21" t="s">
-        <v>10</v>
-      </c>
-      <c r="D21" t="s">
-        <v>49</v>
-      </c>
-      <c r="E21" t="s">
-        <v>9</v>
-      </c>
-      <c r="F21" t="s">
-        <v>9</v>
-      </c>
-      <c r="G21" s="1">
-        <v>17.2</v>
-      </c>
-      <c r="H21">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="22" spans="1:8">
-      <c r="A22" t="s">
-        <v>48</v>
-      </c>
-      <c r="B22" t="s">
-        <v>9</v>
-      </c>
-      <c r="C22" t="s">
-        <v>10</v>
-      </c>
-      <c r="D22" t="s">
-        <v>50</v>
-      </c>
-      <c r="E22" t="s">
-        <v>9</v>
-      </c>
-      <c r="F22" t="s">
-        <v>9</v>
-      </c>
-      <c r="G22" s="1">
-        <v>21.3</v>
-      </c>
-      <c r="H22">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="23" spans="1:8">
-      <c r="A23" t="s">
-        <v>51</v>
-      </c>
-      <c r="B23" t="s">
-        <v>9</v>
-      </c>
-      <c r="C23" t="s">
-        <v>10</v>
-      </c>
-      <c r="D23" t="s">
-        <v>52</v>
-      </c>
-      <c r="E23" t="s">
-        <v>9</v>
-      </c>
-      <c r="F23" t="s">
-        <v>9</v>
-      </c>
-      <c r="G23" s="1">
-        <v>42</v>
-      </c>
-      <c r="H23">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="24" spans="1:8">
-      <c r="A24" t="s">
-        <v>53</v>
-      </c>
-      <c r="B24" t="s">
-        <v>9</v>
-      </c>
-      <c r="C24" t="s">
-        <v>10</v>
-      </c>
-      <c r="D24" t="s">
-        <v>54</v>
-      </c>
-      <c r="E24" t="s">
-        <v>9</v>
-      </c>
-      <c r="F24" t="s">
-        <v>9</v>
-      </c>
-      <c r="G24" s="1">
-        <v>66</v>
-      </c>
-      <c r="H24">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="25" spans="1:8">
-      <c r="A25" t="s">
-        <v>55</v>
-      </c>
-      <c r="B25" t="s">
-        <v>9</v>
-      </c>
-      <c r="C25" t="s">
-        <v>10</v>
-      </c>
-      <c r="D25" t="s">
-        <v>56</v>
-      </c>
-      <c r="E25" t="s">
-        <v>9</v>
-      </c>
-      <c r="F25" t="s">
-        <v>9</v>
-      </c>
-      <c r="G25" s="1">
-        <v>35</v>
-      </c>
-      <c r="H25">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="26" spans="1:8">
-      <c r="A26" t="s">
-        <v>57</v>
-      </c>
-      <c r="B26" t="s">
-        <v>9</v>
-      </c>
-      <c r="C26" t="s">
-        <v>10</v>
-      </c>
-      <c r="D26" t="s">
-        <v>58</v>
-      </c>
-      <c r="E26" t="s">
-        <v>9</v>
-      </c>
-      <c r="F26" t="s">
-        <v>9</v>
-      </c>
-      <c r="G26" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="H26">
-        <v>2</v>
-      </c>
-    </row>
-    <row r="27" spans="1:8">
-      <c r="A27" t="s">
-        <v>57</v>
-      </c>
-      <c r="B27" t="s">
-        <v>9</v>
-      </c>
-      <c r="C27" t="s">
-        <v>10</v>
-      </c>
-      <c r="D27" t="s">
-        <v>60</v>
-      </c>
-      <c r="E27" t="s">
-        <v>9</v>
-      </c>
-      <c r="F27" t="s">
-        <v>9</v>
-      </c>
-      <c r="G27" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="H27">
-        <v>3</v>
-      </c>
-    </row>
-    <row r="28" spans="1:8">
+    <row r="28" spans="1:9">
       <c r="A28" s="2"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A28:H28 G2:G25 D6 D8:D10 D12 D15 D18:D22 D26:D27 A2:B22 B23 A24:B26 B27 A1:H1" numberStoredAsText="1"/>
+    <ignoredError sqref="G28:I28 A24:A26 A1:A22 E26:E27 E18:E22 E15 E12 E8:E10 E6 H2:H25 A28 D28:E28 D1 H1:I1" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
feat(phase-5): magazine panel, data, assets, and docs
- UI: DishInfo, PhotoPanel, MapPanel, RadarChart, CityDetail, global styles

- Data: dishes/restaurants JSON and spreadsheets; photo and sticker assets

- Fallback static maps; storePhotos and formatDishTasteStars helpers

- Docs: PRD updates, archive moves, i18n/UI spec; photo maintenance scripts

- chore: ignore .cursor/ and .compose-row-backup.json

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/src/data/dishes.xlsx
+++ b/src/data/dishes.xlsx
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="442" uniqueCount="174">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="443" uniqueCount="175">
   <si>
     <t>store_slug</t>
   </si>
@@ -192,6 +192,9 @@
   </si>
   <si>
     <t>三文鱼拼甜虾饭</t>
+  </si>
+  <si>
+    <t>作为第一个下单的顾客被送了一份腹肉 耶</t>
   </si>
   <si>
     <t>柚子醋生蚝</t>
@@ -1184,7 +1187,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1197,9 +1200,6 @@
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
       <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
-      <alignment vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="49">
@@ -1734,12 +1734,12 @@
     <col min="3" max="3" width="40.7787610619469" customWidth="1"/>
     <col min="4" max="4" width="30.3362831858407" customWidth="1"/>
     <col min="5" max="5" width="8.53097345132743" customWidth="1"/>
-    <col min="6" max="6" width="82.0442477876106" customWidth="1"/>
-    <col min="7" max="7" width="13.929203539823" customWidth="1"/>
+    <col min="6" max="6" width="46.1769911504425" customWidth="1"/>
+    <col min="7" max="7" width="13.929203539823" hidden="1" customWidth="1"/>
     <col min="8" max="8" width="17.3274336283186" customWidth="1"/>
     <col min="9" max="9" width="6.53097345132743" style="2" customWidth="1"/>
     <col min="10" max="11" width="9.30088495575221" style="2" customWidth="1"/>
-    <col min="12" max="12" width="29.6637168141593" customWidth="1"/>
+    <col min="12" max="12" width="39.3097345132743" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:12">
@@ -2305,7 +2305,7 @@
         <v>4</v>
       </c>
     </row>
-    <row r="17" spans="1:11">
+    <row r="17" spans="1:12">
       <c r="A17" s="1" t="s">
         <v>48</v>
       </c>
@@ -2340,7 +2340,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="18" spans="1:11">
+    <row r="18" spans="1:12">
       <c r="A18" s="1" t="s">
         <v>52</v>
       </c>
@@ -2374,8 +2374,11 @@
       <c r="K18" s="2">
         <v>4</v>
       </c>
-    </row>
-    <row r="19" spans="1:11">
+      <c r="L18" t="s">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="19" spans="1:12">
       <c r="A19" s="1" t="s">
         <v>52</v>
       </c>
@@ -2392,7 +2395,7 @@
         <v>15</v>
       </c>
       <c r="F19" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="G19" t="s">
         <v>14</v>
@@ -2410,12 +2413,12 @@
         <v>1</v>
       </c>
     </row>
-    <row r="20" spans="1:11">
+    <row r="20" spans="1:12">
       <c r="A20" s="1" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="B20" s="4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="C20" t="s">
         <v>14</v>
@@ -2427,7 +2430,7 @@
         <v>15</v>
       </c>
       <c r="F20" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="G20" t="s">
         <v>14</v>
@@ -2445,12 +2448,12 @@
         <v>4</v>
       </c>
     </row>
-    <row r="21" spans="1:11">
+    <row r="21" spans="1:12">
       <c r="A21" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B21" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C21" t="s">
         <v>14</v>
@@ -2462,7 +2465,7 @@
         <v>15</v>
       </c>
       <c r="F21" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="G21" t="s">
         <v>14</v>
@@ -2480,12 +2483,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="22" spans="1:11">
+    <row r="22" spans="1:12">
       <c r="A22" s="1" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="B22" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="C22" t="s">
         <v>14</v>
@@ -2497,7 +2500,7 @@
         <v>15</v>
       </c>
       <c r="F22" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="G22" t="s">
         <v>14</v>
@@ -2515,12 +2518,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="23" spans="1:11">
+    <row r="23" spans="1:12">
       <c r="A23" s="1" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="B23" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="C23" t="s">
         <v>14</v>
@@ -2532,7 +2535,7 @@
         <v>15</v>
       </c>
       <c r="F23" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="G23" t="s">
         <v>14</v>
@@ -2550,12 +2553,12 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:11">
+    <row r="24" spans="1:12">
       <c r="A24" s="1" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="B24" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="C24" t="s">
         <v>14</v>
@@ -2567,7 +2570,7 @@
         <v>15</v>
       </c>
       <c r="F24" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="G24" t="s">
         <v>14</v>
@@ -2585,12 +2588,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="25" spans="1:11">
+    <row r="25" spans="1:12">
       <c r="A25" s="1" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="B25" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="C25" t="s">
         <v>14</v>
@@ -2602,7 +2605,7 @@
         <v>15</v>
       </c>
       <c r="F25" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="G25" t="s">
         <v>14</v>
@@ -2620,12 +2623,12 @@
         <v>3</v>
       </c>
     </row>
-    <row r="26" spans="1:11">
+    <row r="26" spans="1:12">
       <c r="A26" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B26" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C26" t="s">
         <v>14</v>
@@ -2637,7 +2640,7 @@
         <v>15</v>
       </c>
       <c r="F26" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="G26" t="s">
         <v>14</v>
@@ -2646,7 +2649,7 @@
         <v>14</v>
       </c>
       <c r="I26" s="2" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="J26" s="2" t="s">
         <v>18</v>
@@ -2655,12 +2658,12 @@
         <v>2</v>
       </c>
     </row>
-    <row r="27" spans="1:11">
+    <row r="27" spans="1:12">
       <c r="A27" s="1" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="B27" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="C27" t="s">
         <v>14</v>
@@ -2672,7 +2675,7 @@
         <v>15</v>
       </c>
       <c r="F27" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="G27" t="s">
         <v>14</v>
@@ -2681,7 +2684,7 @@
         <v>14</v>
       </c>
       <c r="I27" s="2" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="J27" s="2" t="s">
         <v>18</v>
@@ -2690,357 +2693,357 @@
         <v>3</v>
       </c>
     </row>
-    <row r="28" spans="1:11">
+    <row r="28" spans="1:12">
       <c r="A28" s="1" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B28" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="C28" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="D28" t="s">
         <v>14</v>
       </c>
       <c r="E28" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F28" t="s">
+        <v>83</v>
+      </c>
+      <c r="I28" s="2" t="s">
+        <v>84</v>
+      </c>
+      <c r="J28" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="K28" s="2" t="s">
+        <v>86</v>
+      </c>
+    </row>
+    <row r="29" spans="1:12">
+      <c r="A29" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="B29" t="s">
+        <v>88</v>
+      </c>
+      <c r="C29" t="s">
+        <v>14</v>
+      </c>
+      <c r="D29" t="s">
+        <v>89</v>
+      </c>
+      <c r="E29" t="s">
         <v>82</v>
       </c>
-      <c r="I28" s="2" t="s">
-        <v>83</v>
-      </c>
-      <c r="J28" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="K28" s="2" t="s">
+      <c r="F29" t="s">
+        <v>90</v>
+      </c>
+      <c r="I29" s="2" t="s">
+        <v>91</v>
+      </c>
+      <c r="J29" s="2" t="s">
         <v>85</v>
       </c>
-    </row>
-    <row r="29" spans="1:11">
-      <c r="A29" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="B29" t="s">
-        <v>87</v>
-      </c>
-      <c r="C29" t="s">
-        <v>14</v>
-      </c>
-      <c r="D29" t="s">
-        <v>88</v>
-      </c>
-      <c r="E29" t="s">
-        <v>81</v>
-      </c>
-      <c r="F29" t="s">
-        <v>89</v>
-      </c>
-      <c r="I29" s="2" t="s">
-        <v>90</v>
-      </c>
-      <c r="J29" s="2" t="s">
-        <v>84</v>
-      </c>
       <c r="K29" s="2" t="s">
-        <v>91</v>
-      </c>
-    </row>
-    <row r="30" spans="1:11">
+        <v>92</v>
+      </c>
+    </row>
+    <row r="30" spans="1:12">
       <c r="A30" s="1" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="B30" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="C30" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="D30" t="s">
         <v>14</v>
       </c>
       <c r="E30" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F30" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="I30" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="J30" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K30" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="31" spans="1:11">
+        <v>98</v>
+      </c>
+    </row>
+    <row r="31" spans="1:12">
       <c r="A31" s="1" t="s">
+        <v>99</v>
+      </c>
+      <c r="B31" t="s">
+        <v>100</v>
+      </c>
+      <c r="C31" t="s">
+        <v>101</v>
+      </c>
+      <c r="D31" t="s">
+        <v>14</v>
+      </c>
+      <c r="E31" t="s">
+        <v>82</v>
+      </c>
+      <c r="F31" t="s">
+        <v>102</v>
+      </c>
+      <c r="I31" s="2" t="s">
+        <v>103</v>
+      </c>
+      <c r="J31" s="2" t="s">
+        <v>85</v>
+      </c>
+      <c r="K31" s="2" t="s">
         <v>98</v>
       </c>
-      <c r="B31" t="s">
-        <v>99</v>
-      </c>
-      <c r="C31" t="s">
-        <v>100</v>
-      </c>
-      <c r="D31" t="s">
-        <v>14</v>
-      </c>
-      <c r="E31" t="s">
-        <v>81</v>
-      </c>
-      <c r="F31" t="s">
-        <v>101</v>
-      </c>
-      <c r="I31" s="2" t="s">
-        <v>102</v>
-      </c>
-      <c r="J31" s="2" t="s">
-        <v>84</v>
-      </c>
-      <c r="K31" s="2" t="s">
-        <v>97</v>
-      </c>
-    </row>
-    <row r="32" spans="1:11">
+    </row>
+    <row r="32" spans="1:12">
       <c r="A32" s="1" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="B32" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="C32" t="s">
         <v>14</v>
       </c>
       <c r="D32" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E32" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F32" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="I32" s="2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="J32" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K32" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="33" spans="1:12">
       <c r="A33" s="1" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="B33" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="C33" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="D33" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E33" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F33" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="I33" s="2" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="J33" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K33" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="34" spans="1:12">
       <c r="A34" s="1" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="B34" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="C34" t="s">
         <v>14</v>
       </c>
       <c r="D34" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E34" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F34" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="I34" s="2" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="J34" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K34" s="2" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="35" ht="283.5" spans="1:12">
+        <v>121</v>
+      </c>
+    </row>
+    <row r="35" ht="202.5" spans="1:12">
       <c r="A35" s="1" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="B35" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="C35" t="s">
         <v>14</v>
       </c>
       <c r="D35" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E35" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F35" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="I35" s="2" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="J35" s="2" t="s">
         <v>18</v>
       </c>
       <c r="K35" s="2" t="s">
-        <v>108</v>
-      </c>
-      <c r="L35" s="5" t="s">
-        <v>126</v>
+        <v>109</v>
+      </c>
+      <c r="L35" s="3" t="s">
+        <v>127</v>
       </c>
     </row>
     <row r="36" spans="1:12">
       <c r="A36" s="1" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="C36" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="D36" t="s">
         <v>14</v>
       </c>
       <c r="E36" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F36" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="I36" s="2" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="J36" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K36" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="37" spans="1:12">
       <c r="A37" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B37" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C37" t="s">
         <v>14</v>
       </c>
       <c r="D37" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E37" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F37" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="I37" s="2" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="J37" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K37" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="38" spans="1:12">
       <c r="A38" s="1" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="B38" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="C38" t="s">
         <v>14</v>
       </c>
       <c r="D38" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E38" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F38" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="I38" s="2" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="J38" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K38" s="2" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
     </row>
     <row r="39" spans="1:12">
       <c r="A39" s="1" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="C39" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="D39" t="s">
         <v>14</v>
       </c>
       <c r="E39" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F39" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="I39" s="2" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="J39" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K39" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="40" spans="1:12">
       <c r="A40" s="1" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B40" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="C40" t="s">
         <v>14</v>
@@ -3049,85 +3052,85 @@
         <v>14</v>
       </c>
       <c r="E40" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F40" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="I40" s="2" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="J40" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K40" s="2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
     </row>
     <row r="41" spans="1:12">
       <c r="A41" s="1" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="B41" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="C41" t="s">
         <v>14</v>
       </c>
       <c r="D41" t="s">
-        <v>148</v>
+        <v>149</v>
       </c>
       <c r="E41" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F41" t="s">
-        <v>149</v>
+        <v>150</v>
       </c>
       <c r="I41" s="2" t="s">
-        <v>150</v>
+        <v>151</v>
       </c>
       <c r="J41" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K41" s="2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
     </row>
     <row r="42" spans="1:12">
       <c r="A42" s="1" t="s">
-        <v>151</v>
+        <v>152</v>
       </c>
       <c r="B42" t="s">
-        <v>152</v>
+        <v>153</v>
       </c>
       <c r="C42" t="s">
-        <v>153</v>
+        <v>154</v>
       </c>
       <c r="D42" t="s">
-        <v>154</v>
+        <v>155</v>
       </c>
       <c r="E42" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F42" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="I42" s="2" t="s">
-        <v>156</v>
+        <v>157</v>
       </c>
       <c r="J42" s="2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="K42" s="2" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
     </row>
     <row r="43" spans="1:12">
       <c r="A43" s="1" t="s">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="B43" t="s">
-        <v>158</v>
+        <v>159</v>
       </c>
       <c r="C43" t="s">
         <v>14</v>
@@ -3136,21 +3139,21 @@
         <v>14</v>
       </c>
       <c r="E43" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F43" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="K43" s="2" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
     </row>
     <row r="44" spans="1:12">
       <c r="A44" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B44" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C44" t="s">
         <v>14</v>
@@ -3159,21 +3162,21 @@
         <v>14</v>
       </c>
       <c r="E44" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F44" t="s">
-        <v>162</v>
-      </c>
-      <c r="L44" s="5" t="s">
         <v>163</v>
+      </c>
+      <c r="L44" s="3" t="s">
+        <v>164</v>
       </c>
     </row>
     <row r="45" spans="1:12">
       <c r="A45" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B45" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C45" t="s">
         <v>14</v>
@@ -3182,18 +3185,18 @@
         <v>14</v>
       </c>
       <c r="E45" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F45" t="s">
-        <v>164</v>
+        <v>165</v>
       </c>
     </row>
     <row r="46" spans="1:12">
       <c r="A46" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B46" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C46" t="s">
         <v>14</v>
@@ -3202,18 +3205,18 @@
         <v>14</v>
       </c>
       <c r="E46" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F46" t="s">
-        <v>165</v>
+        <v>166</v>
       </c>
     </row>
     <row r="47" spans="1:12">
       <c r="A47" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B47" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C47" t="s">
         <v>14</v>
@@ -3222,21 +3225,21 @@
         <v>14</v>
       </c>
       <c r="E47" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F47" t="s">
-        <v>166</v>
+        <v>167</v>
       </c>
       <c r="L47" t="s">
-        <v>167</v>
+        <v>168</v>
       </c>
     </row>
     <row r="48" spans="1:12">
       <c r="A48" s="1" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="B48" t="s">
-        <v>161</v>
+        <v>162</v>
       </c>
       <c r="C48" t="s">
         <v>14</v>
@@ -3245,21 +3248,21 @@
         <v>14</v>
       </c>
       <c r="E48" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F48" t="s">
-        <v>168</v>
+        <v>169</v>
       </c>
       <c r="L48" t="s">
-        <v>169</v>
+        <v>170</v>
       </c>
     </row>
     <row r="49" ht="27" spans="1:12">
       <c r="A49" s="1" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="B49" t="s">
-        <v>171</v>
+        <v>172</v>
       </c>
       <c r="C49" t="s">
         <v>14</v>
@@ -3268,13 +3271,13 @@
         <v>14</v>
       </c>
       <c r="E49" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="F49" t="s">
-        <v>172</v>
-      </c>
-      <c r="L49" s="5" t="s">
         <v>173</v>
+      </c>
+      <c r="L49" s="3" t="s">
+        <v>174</v>
       </c>
     </row>
     <row r="50" spans="1:12">
@@ -3284,7 +3287,7 @@
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <headerFooter/>
   <ignoredErrors>
-    <ignoredError sqref="A1:L34 A35:K35 A36:L43 A44:E44 G44:K44 A46:L46 A47:E47 G47:K47 A48:K49 A50:L50" numberStoredAsText="1"/>
+    <ignoredError sqref="A50:L50 A48:K49 G47:K47 A47:E47 A46:L46 G44:K44 A44:E44 A36:L43 A35:K35 A1:L17 A18:K18 A19:L34" numberStoredAsText="1"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>